<commit_message>
added functionality to specify where to store a test file, so the library can be used in many places
</commit_message>
<xml_diff>
--- a/Tests/sample.xlsx
+++ b/Tests/sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wolvey\Desktop\Code\Approvals.Net.Excel\Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FCFF1E-4DE6-4891-A4AF-FD56E381FFD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A1DB41E-8840-43CB-A8E6-5DCCA98BC585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kansilehti" sheetId="23" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="59">
   <si>
     <t>Asiakirja n:o</t>
   </si>
@@ -230,9 +230,6 @@
   </si>
   <si>
     <t>Käyttötapa: Bloo</t>
-  </si>
-  <si>
-    <t>thisbetter break</t>
   </si>
 </sst>
 </file>
@@ -904,16 +901,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -928,6 +915,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
@@ -964,6 +961,15 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
@@ -1008,15 +1014,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
@@ -1679,9 +1676,7 @@
       <c r="X7" s="2"/>
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
-      <c r="AA7" s="42" t="s">
-        <v>48</v>
-      </c>
+      <c r="AA7" s="42"/>
       <c r="AC7" s="2"/>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.2">
@@ -1694,9 +1689,7 @@
       </c>
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
-      <c r="Y8" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="Y8" s="2"/>
       <c r="Z8" s="4"/>
       <c r="AA8" s="43" t="s">
         <v>51</v>
@@ -1951,7 +1944,7 @@
       </c>
     </row>
     <row r="2" spans="1:45" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="117" t="s">
+      <c r="A2" s="123" t="s">
         <v>53</v>
       </c>
       <c r="B2" s="23"/>
@@ -1998,7 +1991,7 @@
       <c r="AO2" s="73"/>
     </row>
     <row r="3" spans="1:45" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="118"/>
+      <c r="A3" s="124"/>
       <c r="B3" s="72"/>
       <c r="C3" s="72"/>
       <c r="D3" s="72"/>
@@ -2041,7 +2034,7 @@
       <c r="AO3" s="74"/>
     </row>
     <row r="4" spans="1:45" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="119"/>
+      <c r="A4" s="125"/>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
       <c r="D4" s="20"/>
@@ -2087,124 +2080,124 @@
       <c r="A5" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="120" t="s">
+      <c r="B5" s="126" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="120" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="H5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="I5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="J5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="K5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="L5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="M5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="N5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="O5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="P5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="R5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="S5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="T5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="U5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="V5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="W5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="X5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AG5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK5" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AL5" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM5" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN5" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO5" s="122" t="s">
+      <c r="C5" s="126" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="J5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="L5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="M5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="N5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="O5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="P5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="R5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="S5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="T5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="U5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="V5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="W5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="X5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK5" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL5" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM5" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN5" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO5" s="118" t="s">
         <v>48</v>
       </c>
       <c r="AP5" s="21"/>
@@ -2216,121 +2209,121 @@
       <c r="B6" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="121" t="s">
+      <c r="C6" s="117" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="F6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="I6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="J6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="K6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="L6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="M6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="N6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="O6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="P6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="R6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="S6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="T6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="U6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="V6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="W6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="X6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AG6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK6" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AL6" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM6" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN6" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO6" s="122" t="s">
+      <c r="D6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="K6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="L6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="M6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="O6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="P6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="R6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="S6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="T6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="U6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="V6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="W6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="X6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK6" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL6" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM6" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN6" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO6" s="118" t="s">
         <v>48</v>
       </c>
       <c r="AP6" s="21"/>
@@ -2342,121 +2335,121 @@
       <c r="B7" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="123" t="s">
+      <c r="C7" s="119" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="F7" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="H7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="I7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="J7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="K7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="L7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="M7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="N7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="O7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="P7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="R7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="S7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="T7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="U7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="V7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="W7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="X7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AG7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH7" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AL7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN7" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO7" s="125" t="s">
+      <c r="D7" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="M7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="N7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="O7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="P7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="R7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="S7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="T7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="U7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="V7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="W7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="X7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH7" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN7" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO7" s="121" t="s">
         <v>48</v>
       </c>
       <c r="AQ7" s="21"/>
@@ -2467,124 +2460,124 @@
       <c r="A8" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="120" t="s">
+      <c r="B8" s="126" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="120" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="J8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="K8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="L8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="M8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="N8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="O8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="P8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="R8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="S8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="T8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="U8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="V8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="W8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="X8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AG8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK8" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AL8" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM8" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN8" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO8" s="122" t="s">
+      <c r="C8" s="126" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="L8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="M8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="N8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="O8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="P8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="R8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="S8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="T8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="U8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="V8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="W8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="X8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK8" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL8" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM8" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN8" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO8" s="118" t="s">
         <v>48</v>
       </c>
       <c r="AP8" s="21"/>
@@ -2596,121 +2589,121 @@
       <c r="B9" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="121" t="s">
+      <c r="C9" s="117" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="I9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="J9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="K9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="L9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="M9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="N9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="O9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="P9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="R9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="S9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="T9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="U9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="V9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="W9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="X9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AG9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK9" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="AL9" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM9" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN9" s="122" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO9" s="122" t="s">
+      <c r="D9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="K9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="L9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="M9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="N9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="O9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="P9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="R9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="S9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="T9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="U9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="V9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="W9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="X9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK9" s="117" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL9" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM9" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN9" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO9" s="118" t="s">
         <v>48</v>
       </c>
       <c r="AP9" s="21"/>
@@ -2722,121 +2715,121 @@
       <c r="B10" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="123" t="s">
+      <c r="C10" s="119" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="G10" s="124" t="s">
-        <v>48</v>
-      </c>
-      <c r="H10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="I10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="J10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="K10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="L10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="M10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="N10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="O10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="P10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="R10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="S10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="T10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="U10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="V10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="W10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="X10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AG10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AH10" s="126" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AL10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN10" s="125" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO10" s="125" t="s">
+      <c r="D10" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="120" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="J10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="K10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="L10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="M10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="N10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="O10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="P10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="R10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="S10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="T10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="U10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="V10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="W10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="X10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH10" s="122" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AM10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN10" s="121" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO10" s="121" t="s">
         <v>48</v>
       </c>
       <c r="AQ10" s="21"/>
@@ -3738,52 +3731,52 @@
       <c r="AO1" s="113"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="V2" s="154" t="s">
+      <c r="V2" s="139" t="s">
         <v>12</v>
       </c>
-      <c r="W2" s="154"/>
-      <c r="X2" s="154"/>
-      <c r="Y2" s="154"/>
-      <c r="Z2" s="154"/>
-      <c r="AA2" s="154"/>
-      <c r="AB2" s="154"/>
-      <c r="AC2" s="154"/>
-      <c r="AD2" s="154"/>
-      <c r="AE2" s="154"/>
-      <c r="AF2" s="154"/>
-      <c r="AG2" s="154"/>
-      <c r="AH2" s="154"/>
-      <c r="AI2" s="154"/>
-      <c r="AJ2" s="154"/>
-      <c r="AK2" s="154"/>
-      <c r="AL2" s="154"/>
-      <c r="AM2" s="154"/>
-      <c r="AN2" s="154"/>
-      <c r="AO2" s="154"/>
+      <c r="W2" s="139"/>
+      <c r="X2" s="139"/>
+      <c r="Y2" s="139"/>
+      <c r="Z2" s="139"/>
+      <c r="AA2" s="139"/>
+      <c r="AB2" s="139"/>
+      <c r="AC2" s="139"/>
+      <c r="AD2" s="139"/>
+      <c r="AE2" s="139"/>
+      <c r="AF2" s="139"/>
+      <c r="AG2" s="139"/>
+      <c r="AH2" s="139"/>
+      <c r="AI2" s="139"/>
+      <c r="AJ2" s="139"/>
+      <c r="AK2" s="139"/>
+      <c r="AL2" s="139"/>
+      <c r="AM2" s="139"/>
+      <c r="AN2" s="139"/>
+      <c r="AO2" s="139"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="V3" s="155" t="s">
+      <c r="V3" s="140" t="s">
         <v>13</v>
       </c>
-      <c r="W3" s="155"/>
-      <c r="X3" s="155"/>
-      <c r="Y3" s="155"/>
-      <c r="Z3" s="155"/>
-      <c r="AA3" s="155"/>
-      <c r="AB3" s="155"/>
-      <c r="AC3" s="155"/>
-      <c r="AD3" s="155"/>
-      <c r="AE3" s="155"/>
-      <c r="AF3" s="155"/>
-      <c r="AG3" s="155"/>
-      <c r="AH3" s="155"/>
-      <c r="AI3" s="155"/>
-      <c r="AJ3" s="155"/>
-      <c r="AK3" s="155"/>
-      <c r="AL3" s="155"/>
-      <c r="AM3" s="155"/>
-      <c r="AN3" s="155"/>
-      <c r="AO3" s="155"/>
+      <c r="W3" s="140"/>
+      <c r="X3" s="140"/>
+      <c r="Y3" s="140"/>
+      <c r="Z3" s="140"/>
+      <c r="AA3" s="140"/>
+      <c r="AB3" s="140"/>
+      <c r="AC3" s="140"/>
+      <c r="AD3" s="140"/>
+      <c r="AE3" s="140"/>
+      <c r="AF3" s="140"/>
+      <c r="AG3" s="140"/>
+      <c r="AH3" s="140"/>
+      <c r="AI3" s="140"/>
+      <c r="AJ3" s="140"/>
+      <c r="AK3" s="140"/>
+      <c r="AL3" s="140"/>
+      <c r="AM3" s="140"/>
+      <c r="AN3" s="140"/>
+      <c r="AO3" s="140"/>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A4" s="107"/>
@@ -3807,28 +3800,28 @@
       <c r="S4" s="107"/>
       <c r="T4" s="107"/>
       <c r="U4" s="107"/>
-      <c r="V4" s="156" t="s">
+      <c r="V4" s="141" t="s">
         <v>14</v>
       </c>
-      <c r="W4" s="156"/>
-      <c r="X4" s="156"/>
-      <c r="Y4" s="156"/>
-      <c r="Z4" s="156"/>
-      <c r="AA4" s="156"/>
-      <c r="AB4" s="156"/>
-      <c r="AC4" s="156"/>
-      <c r="AD4" s="156"/>
-      <c r="AE4" s="156"/>
-      <c r="AF4" s="156"/>
-      <c r="AG4" s="156"/>
-      <c r="AH4" s="156"/>
-      <c r="AI4" s="156"/>
-      <c r="AJ4" s="156"/>
-      <c r="AK4" s="156"/>
-      <c r="AL4" s="156"/>
-      <c r="AM4" s="156"/>
-      <c r="AN4" s="156"/>
-      <c r="AO4" s="156"/>
+      <c r="W4" s="141"/>
+      <c r="X4" s="141"/>
+      <c r="Y4" s="141"/>
+      <c r="Z4" s="141"/>
+      <c r="AA4" s="141"/>
+      <c r="AB4" s="141"/>
+      <c r="AC4" s="141"/>
+      <c r="AD4" s="141"/>
+      <c r="AE4" s="141"/>
+      <c r="AF4" s="141"/>
+      <c r="AG4" s="141"/>
+      <c r="AH4" s="141"/>
+      <c r="AI4" s="141"/>
+      <c r="AJ4" s="141"/>
+      <c r="AK4" s="141"/>
+      <c r="AL4" s="141"/>
+      <c r="AM4" s="141"/>
+      <c r="AN4" s="141"/>
+      <c r="AO4" s="141"/>
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
@@ -4127,10 +4120,10 @@
       <c r="AO11" s="46"/>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A12" s="139" t="s">
+      <c r="A12" s="142" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="140"/>
+      <c r="B12" s="143"/>
       <c r="C12" s="108"/>
       <c r="D12" s="108"/>
       <c r="E12" s="108"/>
@@ -4164,24 +4157,24 @@
       <c r="AE12" s="108"/>
       <c r="AF12" s="108"/>
       <c r="AG12" s="108"/>
-      <c r="AH12" s="145"/>
-      <c r="AI12" s="146"/>
-      <c r="AJ12" s="151" t="s">
+      <c r="AH12" s="148"/>
+      <c r="AI12" s="149"/>
+      <c r="AJ12" s="154" t="s">
         <v>38</v>
       </c>
-      <c r="AK12" s="146"/>
-      <c r="AL12" s="151" t="s">
+      <c r="AK12" s="149"/>
+      <c r="AL12" s="154" t="s">
         <v>22</v>
       </c>
-      <c r="AM12" s="146"/>
-      <c r="AN12" s="151" t="s">
+      <c r="AM12" s="149"/>
+      <c r="AN12" s="154" t="s">
         <v>20</v>
       </c>
-      <c r="AO12" s="146"/>
+      <c r="AO12" s="149"/>
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A13" s="141"/>
-      <c r="B13" s="142"/>
+      <c r="A13" s="144"/>
+      <c r="B13" s="145"/>
       <c r="C13" s="110"/>
       <c r="D13" s="110"/>
       <c r="E13" s="110"/>
@@ -4213,18 +4206,18 @@
       <c r="AE13" s="110"/>
       <c r="AF13" s="110"/>
       <c r="AG13" s="110"/>
-      <c r="AH13" s="147"/>
-      <c r="AI13" s="148"/>
-      <c r="AJ13" s="152"/>
-      <c r="AK13" s="148"/>
-      <c r="AL13" s="152"/>
-      <c r="AM13" s="148"/>
-      <c r="AN13" s="152"/>
-      <c r="AO13" s="148"/>
+      <c r="AH13" s="150"/>
+      <c r="AI13" s="151"/>
+      <c r="AJ13" s="155"/>
+      <c r="AK13" s="151"/>
+      <c r="AL13" s="155"/>
+      <c r="AM13" s="151"/>
+      <c r="AN13" s="155"/>
+      <c r="AO13" s="151"/>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.2">
-      <c r="A14" s="143"/>
-      <c r="B14" s="144"/>
+      <c r="A14" s="146"/>
+      <c r="B14" s="147"/>
       <c r="C14" s="111"/>
       <c r="D14" s="111"/>
       <c r="E14" s="111"/>
@@ -4256,14 +4249,14 @@
       <c r="AE14" s="111"/>
       <c r="AF14" s="111"/>
       <c r="AG14" s="111"/>
-      <c r="AH14" s="149"/>
-      <c r="AI14" s="150"/>
-      <c r="AJ14" s="153"/>
-      <c r="AK14" s="150"/>
-      <c r="AL14" s="153"/>
-      <c r="AM14" s="150"/>
-      <c r="AN14" s="153"/>
-      <c r="AO14" s="150"/>
+      <c r="AH14" s="152"/>
+      <c r="AI14" s="153"/>
+      <c r="AJ14" s="156"/>
+      <c r="AK14" s="153"/>
+      <c r="AL14" s="156"/>
+      <c r="AM14" s="153"/>
+      <c r="AN14" s="156"/>
+      <c r="AO14" s="153"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A15" s="49"/>
@@ -4353,16 +4346,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A12:B14"/>
+    <mergeCell ref="AH12:AI14"/>
+    <mergeCell ref="AJ12:AK14"/>
+    <mergeCell ref="AL12:AM14"/>
+    <mergeCell ref="AN12:AO14"/>
     <mergeCell ref="V1:AO1"/>
     <mergeCell ref="V5:AO5"/>
     <mergeCell ref="V2:AO2"/>
     <mergeCell ref="V3:AO3"/>
     <mergeCell ref="V4:AO4"/>
-    <mergeCell ref="A12:B14"/>
-    <mergeCell ref="AH12:AI14"/>
-    <mergeCell ref="AJ12:AK14"/>
-    <mergeCell ref="AL12:AM14"/>
-    <mergeCell ref="AN12:AO14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4511,12 +4504,12 @@
       <c r="AG3" s="105"/>
       <c r="AH3" s="105"/>
       <c r="AI3" s="105"/>
-      <c r="AJ3" s="147"/>
-      <c r="AK3" s="147"/>
-      <c r="AL3" s="147"/>
-      <c r="AM3" s="147"/>
-      <c r="AN3" s="147"/>
-      <c r="AO3" s="147"/>
+      <c r="AJ3" s="150"/>
+      <c r="AK3" s="150"/>
+      <c r="AL3" s="150"/>
+      <c r="AM3" s="150"/>
+      <c r="AN3" s="150"/>
+      <c r="AO3" s="150"/>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A4" s="159"/>

</xml_diff>